<commit_message>
Refine GANK participation rule
</commit_message>
<xml_diff>
--- a/definitions/dota2_tactical_event_definitions_v1.9_20260609.xlsx
+++ b/definitions/dota2_tactical_event_definitions_v1.9_20260609.xlsx
@@ -1339,12 +1339,12 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>N ? 1?????????? 2 ????????????? 1 ??????</t>
+          <t>N ? 1?????????? 2 ??????????? 1 ??????</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>????/??/?????????????????????????</t>
+          <t>????/??/????????????????????????????</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Add pull lane detection and event rule docs
</commit_message>
<xml_diff>
--- a/definitions/dota2_tactical_event_definitions_v1.9_20260609.xlsx
+++ b/definitions/dota2_tactical_event_definitions_v1.9_20260609.xlsx
@@ -582,7 +582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.75" customWidth="1" min="1" max="1"/>
@@ -828,47 +828,46 @@
       <c r="H6" s="5" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>控符</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>保留</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>A/B：数据库生成+必要时核查</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>符点刷新或符被拾取/罐装/反补时，记录该符点附近双方英雄与最终结果。覆盖普通神符、赏金、水符、护盾、智慧神符；每颗神符只记录一次。</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>match_chat_events 的 RUNE_PICKUP/RUNE_BOTTLE/RUNE_DENY；player_intervals2 位置。同英雄同神符罐装后 90 秒内的拾取日志视为同一颗神符的后续激活，不另记事件。</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>heroes=某符点附近双方英雄；结果=英雄名+拾取/罐装/反补某神符；无结果事件则留空。</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>替代 v1.4 的帮控符和控智慧神符。</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="n"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>对线击杀</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>B：需要人工核查</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>00:20-05:00 内，英雄死亡发生在分路内部的对线期击杀。可作为单杀或小规模冲突的附加标签。</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>combat_logs 英雄死亡；死亡点坐标或死亡英雄最近 player_intervals2 位置；路线判断使用上/中/下路位置口径。</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>追加到战斗标签前；结果列写明路线、次数、死亡时间和死亡英雄。</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>只给单杀、小规模冲突追加；需要标出上路/中路/下路。</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>蹲人</t>
+          <t>控符</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -878,27 +877,27 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>B：需要人工核查</t>
+          <t>A/B：数据库生成+必要时核查</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>英雄在被蹲目标 500-1000 码范围内长时间隐藏或等待，通常在树林、阴影或视野盲区。</t>
+          <t>符点刷新或符被拾取/罐装/反补时，记录该符点附近双方英雄与最终结果。覆盖普通神符、赏金、水符、护盾、智慧神符；每颗神符只记录一次。</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>英雄位置、视野、目标路径可辅助；语义强依赖录像。</t>
+          <t>match_chat_events 的 RUNE_PICKUP/RUNE_BOTTLE/RUNE_DENY；player_intervals2 位置。同英雄同神符罐装后 90 秒内的拾取日志视为同一颗神符的后续激活，不另记事件。</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>被蹲英雄 + 蹲人英雄 + 时间段。</t>
+          <t>heroes=某符点附近双方英雄；结果=英雄名+拾取/罐装/反补某神符；无结果事件则留空。</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>当前建议人工核查。</t>
+          <t>替代 v1.4 的帮控符和控智慧神符。</t>
         </is>
       </c>
       <c r="H8" s="5" t="n"/>
@@ -906,7 +905,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>开雾</t>
+          <t>蹲人</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -921,22 +920,22 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>使用诡计之雾并形成进雾队伍。</t>
+          <t>英雄在被蹲目标 500-1000 码范围内长时间隐藏或等待，通常在树林、阴影或视野盲区。</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>combat_logs 中 item_smoke_of_deceit 使用和 modifier_smoke_of_deceit 添加/移除。</t>
+          <t>英雄位置、视野、目标路径可辅助；语义强依赖录像。</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>使用者 + 进入雾的英雄 + 位置；time_range 从使用到第一个雾状态消失。</t>
+          <t>被蹲英雄 + 蹲人英雄 + 时间段。</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>后续进入同一波雾的英雄也计入。</t>
+          <t>当前建议人工核查。</t>
         </is>
       </c>
       <c r="H9" s="5" t="n"/>
@@ -944,7 +943,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>小规模冲突</t>
+          <t>开雾</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -959,22 +958,22 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>介于单点击杀和团战之间的局部战斗，通常双方各 1-3 人或总人数低于完整团战，但有明确交互和结果。</t>
+          <t>使用诡计之雾并形成进雾队伍。</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>局部伤害/控制/死亡聚类；双方参与者按通用空间/交互规则确认。</t>
+          <t>combat_logs 中 item_smoke_of_deceit 使用和 modifier_smoke_of_deceit 添加/移除。</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>参与双方英雄 + 击杀/死亡变化。</t>
+          <t>使用者 + 进入雾的英雄 + 位置；time_range 从使用到第一个雾状态消失。</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>不能把远端同步消耗并入。</t>
+          <t>后续进入同一波雾的英雄也计入。</t>
         </is>
       </c>
       <c r="H10" s="5" t="n"/>
@@ -982,7 +981,7 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>团战</t>
+          <t>小规模冲突</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -997,22 +996,22 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>双方多名英雄围绕同一局部目标或先手形成持续交战，通常双方各 4 人及以上或达到明确团战强度。</t>
+          <t>介于单点击杀和团战之间的局部战斗，通常双方各 1-3 人或总人数低于完整团战，但有明确交互和结果。</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>伤害、控制、死亡、买活、关键技能、位置聚类。</t>
+          <t>局部伤害/控制/死亡聚类；双方参与者按通用空间/交互规则确认。</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>参与双方英雄 + 击杀/死亡变化 + 关键先手/伤害证据。</t>
+          <t>参与双方英雄 + 击杀/死亡变化。</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>开始/结束遵循团战客观数据标准。</t>
+          <t>不能把远端同步消耗并入。</t>
         </is>
       </c>
       <c r="H11" s="5" t="n"/>
@@ -1020,7 +1019,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>肉山团</t>
+          <t>团战</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
@@ -1035,22 +1034,22 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>肉山存活时，围绕肉山坑附近约 2000 码发生的团战或资源争夺。</t>
+          <t>双方多名英雄围绕同一局部目标或先手形成持续交战，通常双方各 4 人及以上或达到明确团战强度。</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>肉山存活状态、英雄位置、肉山伤害、团战聚类、ROSHAN_KILL/Aegis 事件。</t>
+          <t>伤害、控制、死亡、买活、关键技能、位置聚类。</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>区域 + 参与双方英雄 + 击杀/死亡变化 + 肉山结果。</t>
+          <t>参与双方英雄 + 击杀/死亡变化 + 关键先手/伤害证据。</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>肉山死亡后的后续追击不再误标肉山团。</t>
+          <t>开始/结束遵循团战客观数据标准。</t>
         </is>
       </c>
       <c r="H12" s="5" t="n"/>
@@ -1058,37 +1057,37 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>肉山击杀</t>
+          <t>肉山团</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>新增</t>
+          <t>保留</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>A：数据库可直接生成</t>
+          <t>B：需要人工核查</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>肉山被击杀的资源事件。该事件按阵营归属记录，并合并同一波肉山掉落的获得结果。</t>
+          <t>肉山存活时，围绕肉山坑附近约 2000 码发生的团战或资源争夺。</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>combat_logs roshan_death；match_chat_events ROSHAN_KILL、AEGIS、CHEESE、REFRESHER_SHARD、BANNER_PLANTED 等。</t>
+          <t>肉山存活状态、英雄位置、肉山伤害、团战聚类、ROSHAN_KILL/Aegis 事件。</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>labels=肉山击杀；heroes 输出获得掉落的英雄；结果输出某方击杀肉山以及各英雄获得的盾、奶酪、刷新碎片、战旗等。</t>
+          <t>区域 + 参与双方英雄 + 击杀/死亡变化 + 肉山结果。</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>不再误用 ROSHAN_KILL 的 player/value 字段作为击杀英雄。</t>
+          <t>肉山死亡后的后续追击不再误标肉山团。</t>
         </is>
       </c>
       <c r="H13" s="5" t="n"/>
@@ -1096,37 +1095,37 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>高地团</t>
+          <t>肉山击杀</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>保留</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>B：需要人工核查</t>
+          <t>A：数据库可直接生成</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>一方或双方在高地/基地入口/破路区域发生的团战。</t>
+          <t>肉山被击杀的资源事件。该事件按阵营归属记录，并合并同一波肉山掉落的获得结果。</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>英雄位置、高地坐标、兵营/基地/高地塔事件、战斗聚类。</t>
+          <t>combat_logs roshan_death；match_chat_events ROSHAN_KILL、AEGIS、CHEESE、REFRESHER_SHARD、BANNER_PLANTED 等。</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>区域 + 参与双方英雄 + 击杀/死亡变化。</t>
+          <t>labels=肉山击杀；heroes 输出获得掉落的英雄；结果输出某方击杀肉山以及各英雄获得的盾、奶酪、刷新碎片、战旗等。</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>高地前 poke 与正式开团要拆分。</t>
+          <t>不再误用 ROSHAN_KILL 的 player/value 字段作为击杀英雄。</t>
         </is>
       </c>
       <c r="H14" s="5" t="n"/>
@@ -1134,7 +1133,7 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>守塔团</t>
+          <t>高地团</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -1149,22 +1148,22 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>在一方防御塔附近约 1000 码发生的团战或小规模守塔交战。</t>
+          <t>一方或双方在高地/基地入口/破路区域发生的团战。</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>tower_status_update 塔位置/血量，战斗聚类。</t>
+          <t>英雄位置、高地坐标、兵营/基地/高地塔事件、战斗聚类。</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>区域 + 参与双方英雄 + 击杀/死亡变化 + 防御塔上下文。</t>
+          <t>区域 + 参与双方英雄 + 击杀/死亡变化。</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>守塔上下文是附加标签，可与小规模冲突/团战并存。</t>
+          <t>高地前 poke 与正式开团要拆分。</t>
         </is>
       </c>
       <c r="H15" s="5" t="n"/>
@@ -1172,7 +1171,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>肉山尝试</t>
+          <t>守塔团</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
@@ -1187,22 +1186,22 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>对肉山造成伤害但未完成击杀或未转化为肉山团。</t>
+          <t>在一方防御塔附近约 1000 码发生的团战或小规模守塔交战。</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>combat_logs 对 Roshan 伤害；英雄位置；ROSHAN_KILL 缺失。</t>
+          <t>tower_status_update 塔位置/血量，战斗聚类。</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>伤害英雄 + 第一下伤害到英雄离开肉山区域的时间段。</t>
+          <t>区域 + 参与双方英雄 + 击杀/死亡变化 + 防御塔上下文。</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>若双方围绕肉山开战，优先肉山团。</t>
+          <t>守塔上下文是附加标签，可与小规模冲突/团战并存。</t>
         </is>
       </c>
       <c r="H16" s="5" t="n"/>
@@ -1210,7 +1209,7 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>魔晶团</t>
+          <t>肉山尝试</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -1225,22 +1224,22 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>折磨者/魔晶仍存活时，围绕魔晶区域发生的团战或争夺。</t>
+          <t>对肉山造成伤害但未完成击杀或未转化为肉山团。</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>miniboss damage/kill、英雄位置、团战聚类。</t>
+          <t>combat_logs 对 Roshan 伤害；英雄位置；ROSHAN_KILL 缺失。</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>区域 + 参与双方英雄 + 击杀/死亡变化 + 魔晶归属。</t>
+          <t>伤害英雄 + 第一下伤害到英雄离开肉山区域的时间段。</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>魔晶击杀后的后续交战不再误标魔晶团。</t>
+          <t>若双方围绕肉山开战，优先肉山团。</t>
         </is>
       </c>
       <c r="H17" s="5" t="n"/>
@@ -1248,37 +1247,37 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>资源获得</t>
+          <t>魔晶团</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>新增/合并</t>
+          <t>保留</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>A：数据库可直接生成</t>
+          <t>B：需要人工核查</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>独立记录关键资源时间点，包括击杀肉山、击杀魔晶、获得肉山盾、奶酪、刷新碎片、战旗等。旧抢盾/抢奶/抢刷新并入本标签。</t>
+          <t>折磨者/魔晶仍存活时，围绕魔晶区域发生的团战或争夺。</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>match_chat_events: ROSHAN_KILL、MINIBOSS_KILL、AEGIS、CHEESE、REFRESHER_SHARD、BANNER_PLANTED 等。</t>
+          <t>miniboss damage/kill、英雄位置、团战聚类。</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>获得/击杀资源的英雄或阵营 + 资源类型 + 时间点。</t>
+          <t>区域 + 参与双方英雄 + 击杀/死亡变化 + 魔晶归属。</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>作为资源事实，不强行解释为团战。</t>
+          <t>魔晶击杀后的后续交战不再误标魔晶团。</t>
         </is>
       </c>
       <c r="H18" s="5" t="n"/>
@@ -1286,37 +1285,37 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>带盾阵亡</t>
+          <t>资源获得</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>新增</t>
+          <t>新增/合并</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>A/B：数据库生成+必要时核查</t>
+          <t>A：数据库可直接生成</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>携带不朽盾的英雄阵亡时独立记录；团战死亡列表中也要标注带盾阵亡。</t>
+          <t>独立记录关键资源时间点，包括击杀肉山、击杀魔晶、获得肉山盾、奶酪、刷新碎片、战旗等。旧抢盾/抢奶/抢刷新并入本标签。</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Aegis 获得事件、英雄死亡事件、复活/盾消耗上下文。</t>
+          <t>match_chat_events: ROSHAN_KILL、MINIBOSS_KILL、AEGIS、CHEESE、REFRESHER_SHARD、BANNER_PLANTED 等。</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>带盾英雄 + 阵亡时间 + 相关战斗/位置。</t>
+          <t>获得/击杀资源的英雄或阵营 + 资源类型 + 时间点。</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>用于区分普通死亡和战略资源消耗。</t>
+          <t>作为资源事实，不强行解释为团战。</t>
         </is>
       </c>
       <c r="H19" s="5" t="n"/>
@@ -1324,40 +1323,115 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
+          <t>带盾阵亡</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>A/B：数据库生成+必要时核查</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>携带不朽盾的英雄阵亡时独立记录；团战死亡列表中也要标注带盾阵亡。</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Aegis 获得事件、英雄死亡事件、复活/盾消耗上下文。</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>带盾英雄 + 阵亡时间 + 相关战斗/位置。</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>用于区分普通死亡和战略资源消耗。</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
           <t>GANK</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>??</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>B???????</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>N ? 1?????????? 2 ??????????? 1 ??????</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>????/??/????????????????????????????</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="F21" s="5" t="inlineStr">
         <is>
           <t>gank ??? + ???? + ??/?????</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="G21" s="5" t="inlineStr">
         <is>
           <t>????????????????????????????</t>
         </is>
       </c>
-      <c r="H20" s="5" t="inlineStr"/>
+      <c r="H21" s="5" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>单杀</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>B：需要人工核查</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>1v1 战斗聚类中双方各只有 1 名英雄参与，并且其中一方英雄阵亡。</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>combat_logs 中英雄对英雄伤害、控制和死亡；player_intervals2 可辅助确认位置；排除幻象、召唤物独立误归因和远端无关伤害。</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>双方英雄 + 击杀比分 + 死亡英雄与时间。</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>不追加守塔团、肉山团等团队上下文；无英雄死亡的 1v1 消耗不输出单杀。</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update tactical event pipeline outputs
</commit_message>
<xml_diff>
--- a/definitions/dota2_tactical_event_definitions_v1.9_20260609.xlsx
+++ b/definitions/dota2_tactical_event_definitions_v1.9_20260609.xlsx
@@ -1171,7 +1171,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>守塔团</t>
+          <t>塔下</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>不追加守塔团、肉山团等团队上下文；无英雄死亡的 1v1 消耗不输出单杀。</t>
+          <t>不追加塔下、肉山团等团队上下文；无英雄死亡的 1v1 消耗不输出单杀。</t>
         </is>
       </c>
     </row>
@@ -1505,7 +1505,7 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>小规模冲突、团战、肉山团、高地团、守塔团、魔晶团</t>
+          <t>小规模冲突、团战、肉山团、高地团、塔下、魔晶团</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -1841,7 +1841,7 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>小规模冲突、团战、肉山团、高地团、守塔团、魔晶团</t>
+          <t>小规模冲突、团战、肉山团、高地团、塔下、魔晶团</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>小规模冲突、团战、肉山团、高地团、守塔团、魔晶团</t>
+          <t>小规模冲突、团战、肉山团、高地团、塔下、魔晶团</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -1981,7 +1981,7 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>小规模冲突、团战、肉山团、高地团、守塔团、魔晶团</t>
+          <t>小规模冲突、团战、肉山团、高地团、塔下、魔晶团</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -2009,7 +2009,7 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>小规模冲突、团战、肉山团、高地团、守塔团、魔晶团</t>
+          <t>小规模冲突、团战、肉山团、高地团、塔下、魔晶团</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>多标签用 / 分隔，例如 小规模冲突 / 守塔团</t>
+          <t>多标签用 / 分隔，例如 小规模冲突 / 塔下</t>
         </is>
       </c>
       <c r="E4" s="5" t="n"/>

</xml_diff>